<commit_message>
Updated sign in automation code
</commit_message>
<xml_diff>
--- a/src/test/resources/DaikinorgaDatas.xlsx
+++ b/src/test/resources/DaikinorgaDatas.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\x16\eclipse-workspace\claimManagement\src\test\resources\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/2a1d2811b9ce554d/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1B72A65-622B-42DC-82EE-0A4255AA39F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="571" documentId="8_{E84906A2-3816-4B9B-BDA1-728A7EC25049}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C420A4E1-B119-4CDE-BFB1-690B4B5E2ECB}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" firstSheet="10" activeTab="13" xr2:uid="{2D8CCF5D-6ECB-41C4-80C4-99CF4F2974CD}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{2D8CCF5D-6ECB-41C4-80C4-99CF4F2974CD}"/>
   </bookViews>
   <sheets>
     <sheet name="Signin" sheetId="1" r:id="rId1"/>
@@ -52,7 +52,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="882" uniqueCount="224">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="852" uniqueCount="207">
   <si>
     <t>UserName</t>
   </si>
@@ -468,54 +468,6 @@
     <t>20 Jul 2026</t>
   </si>
   <si>
-    <t>Gopi007</t>
-  </si>
-  <si>
-    <t>Vijay1</t>
-  </si>
-  <si>
-    <t>Devi1</t>
-  </si>
-  <si>
-    <t>Dhiviya1</t>
-  </si>
-  <si>
-    <t>Kesaven1</t>
-  </si>
-  <si>
-    <t>Ruthra1</t>
-  </si>
-  <si>
-    <t>Nedu1</t>
-  </si>
-  <si>
-    <t>PonKarthick1</t>
-  </si>
-  <si>
-    <t>Hari1</t>
-  </si>
-  <si>
-    <t>Sabari1</t>
-  </si>
-  <si>
-    <t>Asma1</t>
-  </si>
-  <si>
-    <t>Sriram1</t>
-  </si>
-  <si>
-    <t>Dhanish1</t>
-  </si>
-  <si>
-    <t>Karthikeyan1</t>
-  </si>
-  <si>
-    <t>Oviya1</t>
-  </si>
-  <si>
-    <t>Suvetha</t>
-  </si>
-  <si>
     <t>ann</t>
   </si>
   <si>
@@ -721,9 +673,6 @@
   </si>
   <si>
     <t>01-07-2026</t>
-  </si>
-  <si>
-    <t>30-06-2026</t>
   </si>
 </sst>
 </file>
@@ -795,6 +744,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1110,476 +1063,186 @@
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A2" s="3" t="s">
-        <v>156</v>
+      <c r="A2" t="s">
+        <v>138</v>
       </c>
       <c r="B2" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A3" s="3" t="s">
-        <v>157</v>
-      </c>
-      <c r="B3" t="s">
-        <v>2</v>
-      </c>
+      <c r="A3"/>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A4" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="B4" t="s">
-        <v>2</v>
-      </c>
+      <c r="A4"/>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A5" s="3" t="s">
-        <v>158</v>
-      </c>
-      <c r="B5" t="s">
-        <v>2</v>
-      </c>
+      <c r="A5"/>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A6" s="3" t="s">
-        <v>159</v>
-      </c>
-      <c r="B6" t="s">
-        <v>2</v>
-      </c>
+      <c r="A6"/>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A7" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="B7" t="s">
-        <v>2</v>
-      </c>
+      <c r="A7"/>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A8" s="3" t="s">
-        <v>160</v>
-      </c>
-      <c r="B8" t="s">
-        <v>2</v>
-      </c>
+      <c r="A8"/>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A9" s="3" t="s">
-        <v>161</v>
-      </c>
-      <c r="B9" t="s">
-        <v>2</v>
-      </c>
+      <c r="A9"/>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A10" s="3" t="s">
-        <v>162</v>
-      </c>
-      <c r="B10" t="s">
-        <v>2</v>
-      </c>
+      <c r="A10"/>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A11" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="B11" t="s">
-        <v>2</v>
-      </c>
+      <c r="A11"/>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A12" s="3" t="s">
-        <v>163</v>
-      </c>
-      <c r="B12" t="s">
-        <v>2</v>
-      </c>
+      <c r="A12"/>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A13" s="3" t="s">
-        <v>164</v>
-      </c>
-      <c r="B13" t="s">
-        <v>2</v>
-      </c>
+      <c r="A13"/>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A14" s="3" t="s">
-        <v>165</v>
-      </c>
-      <c r="B14" t="s">
-        <v>2</v>
-      </c>
+      <c r="A14"/>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A15" s="3" t="s">
-        <v>166</v>
-      </c>
-      <c r="B15" t="s">
-        <v>2</v>
-      </c>
+      <c r="A15"/>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A16" s="3" t="s">
-        <v>167</v>
-      </c>
-      <c r="B16" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A17" s="3" t="s">
-        <v>168</v>
-      </c>
-      <c r="B17" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A18" s="3" t="s">
-        <v>169</v>
-      </c>
-      <c r="B18" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A19" s="3" t="s">
-        <v>170</v>
-      </c>
-      <c r="B19" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A20" s="3" t="s">
-        <v>155</v>
-      </c>
-      <c r="B20" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A21" s="3" t="s">
-        <v>171</v>
-      </c>
-      <c r="B21" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A22" s="3" t="s">
-        <v>172</v>
-      </c>
-      <c r="B22" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A23" s="3" t="s">
-        <v>173</v>
-      </c>
-      <c r="B23" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A24" s="3" t="s">
-        <v>174</v>
-      </c>
-      <c r="B24" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A25" s="3" t="s">
-        <v>175</v>
-      </c>
-      <c r="B25" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A26" s="3" t="s">
-        <v>176</v>
-      </c>
-      <c r="B26" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A27" s="3" t="s">
-        <v>177</v>
-      </c>
-      <c r="B27" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A28" s="3" t="s">
-        <v>178</v>
-      </c>
-      <c r="B28" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A29" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="B29" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A30" s="3" t="s">
-        <v>180</v>
-      </c>
-      <c r="B30" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A31" s="3" t="s">
-        <v>181</v>
-      </c>
-      <c r="B31" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A32" s="3" t="s">
-        <v>182</v>
-      </c>
-      <c r="B32" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A33" s="3" t="s">
-        <v>183</v>
-      </c>
-      <c r="B33" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A34" s="3" t="s">
-        <v>184</v>
-      </c>
-      <c r="B34" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A35" s="3" t="s">
-        <v>185</v>
-      </c>
-      <c r="B35" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A36" s="3" t="s">
-        <v>186</v>
-      </c>
-      <c r="B36" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A37" s="3" t="s">
-        <v>187</v>
-      </c>
-      <c r="B37" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A38" s="3" t="s">
-        <v>188</v>
-      </c>
-      <c r="B38" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A39" s="3" t="s">
-        <v>189</v>
-      </c>
-      <c r="B39" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A40" s="3" t="s">
-        <v>190</v>
-      </c>
-      <c r="B40" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A41" s="3" t="s">
-        <v>191</v>
-      </c>
-      <c r="B41" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A42" s="3" t="s">
-        <v>192</v>
-      </c>
-      <c r="B42" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A43" s="3" t="s">
-        <v>193</v>
-      </c>
-      <c r="B43" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A44" s="3" t="s">
-        <v>194</v>
-      </c>
-      <c r="B44" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A45" s="3" t="s">
-        <v>195</v>
-      </c>
-      <c r="B45" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A46" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="B46" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="47" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A47" s="3" t="s">
-        <v>196</v>
-      </c>
-      <c r="B47" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="48" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A48" s="3" t="s">
-        <v>197</v>
-      </c>
-      <c r="B48" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="49" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A49" s="3" t="s">
-        <v>198</v>
-      </c>
-      <c r="B49" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="50" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A50" s="3" t="s">
-        <v>199</v>
-      </c>
-      <c r="B50" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="51" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A51" s="3" t="s">
-        <v>200</v>
-      </c>
-      <c r="B51" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="52" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A52" s="3" t="s">
-        <v>201</v>
-      </c>
-      <c r="B52" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="53" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A53" s="3" t="s">
-        <v>202</v>
-      </c>
-      <c r="B53" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="54" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A54" s="3" t="s">
-        <v>203</v>
-      </c>
-      <c r="B54" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="55" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A55" s="3" t="s">
-        <v>204</v>
-      </c>
-      <c r="B55" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="56" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A56" s="3" t="s">
-        <v>205</v>
-      </c>
-      <c r="B56" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="57" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A57" s="3" t="s">
-        <v>206</v>
-      </c>
-      <c r="B57" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="58" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A58" s="3" t="s">
-        <v>207</v>
-      </c>
-      <c r="B58" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="59" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A59" s="3" t="s">
-        <v>208</v>
-      </c>
-      <c r="B59" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="60" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A60" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="B60" t="s">
-        <v>2</v>
-      </c>
+      <c r="A16"/>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A17"/>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A18"/>
+    </row>
+    <row r="19" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A19"/>
+    </row>
+    <row r="20" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A20"/>
+    </row>
+    <row r="21" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A21"/>
+    </row>
+    <row r="22" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A22"/>
+    </row>
+    <row r="23" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A23"/>
+    </row>
+    <row r="24" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A24"/>
+    </row>
+    <row r="25" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A25"/>
+    </row>
+    <row r="26" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A26"/>
+    </row>
+    <row r="27" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A27"/>
+    </row>
+    <row r="28" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A28"/>
+    </row>
+    <row r="29" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A29"/>
+    </row>
+    <row r="30" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A30"/>
+    </row>
+    <row r="31" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A31"/>
+    </row>
+    <row r="32" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A32"/>
+    </row>
+    <row r="33" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A33"/>
+    </row>
+    <row r="34" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A34"/>
+    </row>
+    <row r="35" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A35"/>
+    </row>
+    <row r="36" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A36"/>
+    </row>
+    <row r="37" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A37"/>
+    </row>
+    <row r="38" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A38"/>
+    </row>
+    <row r="39" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A39"/>
+    </row>
+    <row r="40" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A40"/>
+    </row>
+    <row r="41" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A41"/>
+    </row>
+    <row r="42" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A42"/>
+    </row>
+    <row r="43" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A43"/>
+    </row>
+    <row r="44" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A44"/>
+    </row>
+    <row r="45" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A45"/>
+    </row>
+    <row r="46" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A46"/>
+    </row>
+    <row r="47" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A47"/>
+    </row>
+    <row r="48" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A48"/>
+    </row>
+    <row r="49" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A49"/>
+    </row>
+    <row r="50" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A50"/>
+    </row>
+    <row r="51" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A51"/>
+    </row>
+    <row r="52" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A52"/>
+    </row>
+    <row r="53" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A53"/>
+    </row>
+    <row r="54" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A54"/>
+    </row>
+    <row r="55" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A55"/>
+    </row>
+    <row r="56" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A56"/>
+    </row>
+    <row r="57" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A57"/>
+    </row>
+    <row r="58" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A58"/>
+    </row>
+    <row r="59" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A59"/>
+    </row>
+    <row r="60" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A60"/>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
@@ -1947,13 +1610,13 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>154</v>
+        <v>138</v>
       </c>
       <c r="B2" t="s">
         <v>2</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>223</v>
+        <v>100</v>
       </c>
       <c r="D2" s="1" t="s">
         <v>16</v>
@@ -1968,7 +1631,6 @@
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -2006,13 +1668,13 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>154</v>
+        <v>138</v>
       </c>
       <c r="B2" t="s">
         <v>2</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>223</v>
+        <v>100</v>
       </c>
       <c r="D2" s="1" t="s">
         <v>33</v>
@@ -2059,13 +1721,13 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>154</v>
+        <v>138</v>
       </c>
       <c r="B2" t="s">
         <v>2</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>222</v>
+        <v>206</v>
       </c>
       <c r="D2" s="1" t="s">
         <v>46</v>
@@ -2112,7 +1774,7 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>154</v>
+        <v>138</v>
       </c>
       <c r="B2" t="s">
         <v>2</v>
@@ -2182,13 +1844,13 @@
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
-        <v>156</v>
+        <v>140</v>
       </c>
       <c r="B2" t="s">
         <v>2</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>215</v>
+        <v>199</v>
       </c>
       <c r="D2" s="1" t="s">
         <v>13</v>
@@ -2211,13 +1873,13 @@
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
-        <v>157</v>
+        <v>141</v>
       </c>
       <c r="B3" t="s">
         <v>2</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>215</v>
+        <v>199</v>
       </c>
       <c r="D3" s="1" t="s">
         <v>13</v>
@@ -2246,7 +1908,7 @@
         <v>2</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>215</v>
+        <v>199</v>
       </c>
       <c r="D4" s="1" t="s">
         <v>13</v>
@@ -2269,13 +1931,13 @@
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
-        <v>158</v>
+        <v>142</v>
       </c>
       <c r="B5" t="s">
         <v>2</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>215</v>
+        <v>199</v>
       </c>
       <c r="D5" s="1" t="s">
         <v>13</v>
@@ -2298,13 +1960,13 @@
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A6" s="3" t="s">
-        <v>159</v>
+        <v>143</v>
       </c>
       <c r="B6" t="s">
         <v>2</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>215</v>
+        <v>199</v>
       </c>
       <c r="D6" s="1" t="s">
         <v>13</v>
@@ -2333,7 +1995,7 @@
         <v>2</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>215</v>
+        <v>199</v>
       </c>
       <c r="D7" s="1" t="s">
         <v>13</v>
@@ -2431,13 +2093,13 @@
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
-        <v>156</v>
+        <v>140</v>
       </c>
       <c r="B2" t="s">
         <v>2</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>215</v>
+        <v>199</v>
       </c>
       <c r="D2" s="1" t="s">
         <v>13</v>
@@ -2478,13 +2140,13 @@
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
-        <v>157</v>
+        <v>141</v>
       </c>
       <c r="B3" t="s">
         <v>2</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>215</v>
+        <v>199</v>
       </c>
       <c r="D3" s="1" t="s">
         <v>13</v>
@@ -2531,7 +2193,7 @@
         <v>2</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>215</v>
+        <v>199</v>
       </c>
       <c r="D4" s="1" t="s">
         <v>13</v>
@@ -2572,13 +2234,13 @@
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
-        <v>158</v>
+        <v>142</v>
       </c>
       <c r="B5" t="s">
         <v>2</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>215</v>
+        <v>199</v>
       </c>
       <c r="D5" s="1" t="s">
         <v>13</v>
@@ -2619,13 +2281,13 @@
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A6" s="3" t="s">
-        <v>159</v>
+        <v>143</v>
       </c>
       <c r="B6" t="s">
         <v>2</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>215</v>
+        <v>199</v>
       </c>
       <c r="D6" s="1" t="s">
         <v>13</v>
@@ -2672,7 +2334,7 @@
         <v>2</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>215</v>
+        <v>199</v>
       </c>
       <c r="D7" s="1" t="s">
         <v>13</v>
@@ -2746,16 +2408,16 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>218</v>
+        <v>202</v>
       </c>
       <c r="B2" t="s">
         <v>2</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>215</v>
+        <v>199</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>215</v>
+        <v>199</v>
       </c>
       <c r="E2" t="s">
         <v>56</v>
@@ -2763,16 +2425,16 @@
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>216</v>
+        <v>200</v>
       </c>
       <c r="B3" t="s">
         <v>2</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>215</v>
+        <v>199</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>215</v>
+        <v>199</v>
       </c>
       <c r="E3" t="s">
         <v>57</v>
@@ -2780,16 +2442,16 @@
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>217</v>
+        <v>201</v>
       </c>
       <c r="B4" t="s">
         <v>2</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>215</v>
+        <v>199</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>215</v>
+        <v>199</v>
       </c>
       <c r="E4" t="s">
         <v>56</v>
@@ -2797,16 +2459,16 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>219</v>
+        <v>203</v>
       </c>
       <c r="B5" t="s">
         <v>2</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>215</v>
+        <v>199</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>215</v>
+        <v>199</v>
       </c>
       <c r="E5" t="s">
         <v>57</v>
@@ -2814,16 +2476,16 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>220</v>
+        <v>204</v>
       </c>
       <c r="B6" t="s">
         <v>2</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>215</v>
+        <v>199</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>215</v>
+        <v>199</v>
       </c>
       <c r="E6" t="s">
         <v>56</v>
@@ -2831,16 +2493,16 @@
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>221</v>
+        <v>205</v>
       </c>
       <c r="B7" t="s">
         <v>2</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>215</v>
+        <v>199</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>215</v>
+        <v>199</v>
       </c>
       <c r="E7" t="s">
         <v>57</v>
@@ -2854,15 +2516,15 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{232400F6-BD8B-483F-A78F-DD3414833EDF}">
-  <dimension ref="A1:B17"/>
+  <dimension ref="A1:B60"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="14.6640625" customWidth="1"/>
+    <col min="1" max="1" width="14.6640625" style="2" customWidth="1"/>
     <col min="2" max="2" width="14.88671875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
@@ -2870,130 +2532,474 @@
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>138</v>
+      <c r="A2" s="3" t="s">
+        <v>140</v>
       </c>
       <c r="B2" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
+      <c r="A3" s="3" t="s">
+        <v>141</v>
+      </c>
+      <c r="B3" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A4" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="B4" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A5" s="3" t="s">
+        <v>142</v>
+      </c>
+      <c r="B5" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A6" s="3" t="s">
+        <v>143</v>
+      </c>
+      <c r="B6" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A7" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="B7" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A8" s="3" t="s">
+        <v>144</v>
+      </c>
+      <c r="B8" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A9" s="3" t="s">
+        <v>145</v>
+      </c>
+      <c r="B9" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A10" s="3" t="s">
+        <v>146</v>
+      </c>
+      <c r="B10" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A11" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="B11" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A12" s="3" t="s">
+        <v>147</v>
+      </c>
+      <c r="B12" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A13" s="3" t="s">
+        <v>148</v>
+      </c>
+      <c r="B13" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A14" s="3" t="s">
+        <v>149</v>
+      </c>
+      <c r="B14" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A15" s="3" t="s">
+        <v>150</v>
+      </c>
+      <c r="B15" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A16" s="3" t="s">
+        <v>151</v>
+      </c>
+      <c r="B16" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A17" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="B17" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A18" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="B18" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A19" s="3" t="s">
+        <v>154</v>
+      </c>
+      <c r="B19" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A20" s="3" t="s">
         <v>139</v>
       </c>
-      <c r="B3" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>140</v>
-      </c>
-      <c r="B4" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>141</v>
-      </c>
-      <c r="B5" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
-        <v>142</v>
-      </c>
-      <c r="B6" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
-        <v>143</v>
-      </c>
-      <c r="B7" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
-        <v>144</v>
-      </c>
-      <c r="B8" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
-        <v>145</v>
-      </c>
-      <c r="B9" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A10" t="s">
-        <v>146</v>
-      </c>
-      <c r="B10" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A11" t="s">
-        <v>147</v>
-      </c>
-      <c r="B11" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A12" t="s">
-        <v>148</v>
-      </c>
-      <c r="B12" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A13" t="s">
-        <v>149</v>
-      </c>
-      <c r="B13" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A14" t="s">
-        <v>150</v>
-      </c>
-      <c r="B14" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A15" t="s">
-        <v>151</v>
-      </c>
-      <c r="B15" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A16" t="s">
-        <v>152</v>
-      </c>
-      <c r="B16" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A17" t="s">
-        <v>153</v>
-      </c>
-      <c r="B17" t="s">
+      <c r="B20" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A21" s="3" t="s">
+        <v>155</v>
+      </c>
+      <c r="B21" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A22" s="3" t="s">
+        <v>156</v>
+      </c>
+      <c r="B22" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A23" s="3" t="s">
+        <v>157</v>
+      </c>
+      <c r="B23" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A24" s="3" t="s">
+        <v>158</v>
+      </c>
+      <c r="B24" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A25" s="3" t="s">
+        <v>159</v>
+      </c>
+      <c r="B25" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A26" s="3" t="s">
+        <v>160</v>
+      </c>
+      <c r="B26" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A27" s="3" t="s">
+        <v>161</v>
+      </c>
+      <c r="B27" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A28" s="3" t="s">
+        <v>162</v>
+      </c>
+      <c r="B28" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A29" s="3" t="s">
+        <v>163</v>
+      </c>
+      <c r="B29" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A30" s="3" t="s">
+        <v>164</v>
+      </c>
+      <c r="B30" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A31" s="3" t="s">
+        <v>165</v>
+      </c>
+      <c r="B31" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A32" s="3" t="s">
+        <v>166</v>
+      </c>
+      <c r="B32" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A33" s="3" t="s">
+        <v>167</v>
+      </c>
+      <c r="B33" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A34" s="3" t="s">
+        <v>168</v>
+      </c>
+      <c r="B34" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A35" s="3" t="s">
+        <v>169</v>
+      </c>
+      <c r="B35" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A36" s="3" t="s">
+        <v>170</v>
+      </c>
+      <c r="B36" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A37" s="3" t="s">
+        <v>171</v>
+      </c>
+      <c r="B37" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A38" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="B38" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A39" s="3" t="s">
+        <v>173</v>
+      </c>
+      <c r="B39" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A40" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="B40" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A41" s="3" t="s">
+        <v>175</v>
+      </c>
+      <c r="B41" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="42" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A42" s="3" t="s">
+        <v>176</v>
+      </c>
+      <c r="B42" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="43" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A43" s="3" t="s">
+        <v>177</v>
+      </c>
+      <c r="B43" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="44" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A44" s="3" t="s">
+        <v>178</v>
+      </c>
+      <c r="B44" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="45" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A45" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="B45" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="46" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A46" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B46" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="47" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A47" s="3" t="s">
+        <v>180</v>
+      </c>
+      <c r="B47" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="48" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A48" s="3" t="s">
+        <v>181</v>
+      </c>
+      <c r="B48" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="49" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A49" s="3" t="s">
+        <v>182</v>
+      </c>
+      <c r="B49" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="50" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A50" s="3" t="s">
+        <v>183</v>
+      </c>
+      <c r="B50" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="51" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A51" s="3" t="s">
+        <v>184</v>
+      </c>
+      <c r="B51" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="52" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A52" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="B52" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="53" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A53" s="3" t="s">
+        <v>186</v>
+      </c>
+      <c r="B53" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="54" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A54" s="3" t="s">
+        <v>187</v>
+      </c>
+      <c r="B54" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="55" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A55" s="3" t="s">
+        <v>188</v>
+      </c>
+      <c r="B55" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="56" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A56" s="3" t="s">
+        <v>189</v>
+      </c>
+      <c r="B56" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="57" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A57" s="3" t="s">
+        <v>190</v>
+      </c>
+      <c r="B57" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="58" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A58" s="3" t="s">
+        <v>191</v>
+      </c>
+      <c r="B58" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="59" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A59" s="3" t="s">
+        <v>192</v>
+      </c>
+      <c r="B59" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="60" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A60" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B60" t="s">
         <v>2</v>
       </c>
     </row>
@@ -3025,24 +3031,24 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
-        <v>156</v>
+        <v>140</v>
       </c>
       <c r="B2" t="s">
         <v>2</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>215</v>
+        <v>199</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
-        <v>157</v>
+        <v>141</v>
       </c>
       <c r="B3" t="s">
         <v>2</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>215</v>
+        <v>199</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
@@ -3053,29 +3059,29 @@
         <v>2</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>215</v>
+        <v>199</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
-        <v>158</v>
+        <v>142</v>
       </c>
       <c r="B5" t="s">
         <v>2</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>215</v>
+        <v>199</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" s="3" t="s">
-        <v>159</v>
+        <v>143</v>
       </c>
       <c r="B6" t="s">
         <v>2</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>215</v>
+        <v>199</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
@@ -3086,7 +3092,7 @@
         <v>2</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>215</v>
+        <v>199</v>
       </c>
     </row>
   </sheetData>
@@ -3121,86 +3127,86 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>209</v>
+        <v>193</v>
       </c>
       <c r="B2" t="s">
         <v>2</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>215</v>
+        <v>199</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>215</v>
+        <v>199</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>210</v>
+        <v>194</v>
       </c>
       <c r="B3" t="s">
         <v>2</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>215</v>
+        <v>199</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>215</v>
+        <v>199</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>211</v>
+        <v>195</v>
       </c>
       <c r="B4" t="s">
         <v>2</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>215</v>
+        <v>199</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>215</v>
+        <v>199</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>212</v>
+        <v>196</v>
       </c>
       <c r="B5" t="s">
         <v>2</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>215</v>
+        <v>199</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>215</v>
+        <v>199</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>213</v>
+        <v>197</v>
       </c>
       <c r="B6" t="s">
         <v>2</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>215</v>
+        <v>199</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>215</v>
+        <v>199</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>214</v>
+        <v>198</v>
       </c>
       <c r="B7" t="s">
         <v>2</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>215</v>
+        <v>199</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>215</v>
+        <v>199</v>
       </c>
     </row>
   </sheetData>
@@ -3321,30 +3327,30 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
-        <v>156</v>
+        <v>140</v>
       </c>
       <c r="B2" t="s">
         <v>2</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>215</v>
+        <v>199</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>215</v>
+        <v>199</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
-        <v>157</v>
+        <v>141</v>
       </c>
       <c r="B3" t="s">
         <v>2</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>215</v>
+        <v>199</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>215</v>
+        <v>199</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
@@ -3355,38 +3361,38 @@
         <v>2</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>215</v>
+        <v>199</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>215</v>
+        <v>199</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
-        <v>158</v>
+        <v>142</v>
       </c>
       <c r="B5" t="s">
         <v>2</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>215</v>
+        <v>199</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>215</v>
+        <v>199</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" s="3" t="s">
-        <v>159</v>
+        <v>143</v>
       </c>
       <c r="B6" t="s">
         <v>2</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>215</v>
+        <v>199</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>215</v>
+        <v>199</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.3">
@@ -3397,10 +3403,10 @@
         <v>2</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>215</v>
+        <v>199</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>215</v>
+        <v>199</v>
       </c>
     </row>
   </sheetData>
@@ -3440,16 +3446,16 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
-        <v>156</v>
+        <v>140</v>
       </c>
       <c r="B2" t="s">
         <v>2</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>215</v>
+        <v>199</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>215</v>
+        <v>199</v>
       </c>
       <c r="E2" s="1">
         <v>10</v>
@@ -3457,16 +3463,16 @@
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
-        <v>157</v>
+        <v>141</v>
       </c>
       <c r="B3" t="s">
         <v>2</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>215</v>
+        <v>199</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>215</v>
+        <v>199</v>
       </c>
       <c r="E3" s="1">
         <v>11</v>
@@ -3480,10 +3486,10 @@
         <v>2</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>215</v>
+        <v>199</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>215</v>
+        <v>199</v>
       </c>
       <c r="E4" s="1">
         <v>12</v>
@@ -3491,16 +3497,16 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
-        <v>158</v>
+        <v>142</v>
       </c>
       <c r="B5" t="s">
         <v>2</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>215</v>
+        <v>199</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>215</v>
+        <v>199</v>
       </c>
       <c r="E5" s="1">
         <v>13</v>
@@ -3508,16 +3514,16 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" s="3" t="s">
-        <v>159</v>
+        <v>143</v>
       </c>
       <c r="B6" t="s">
         <v>2</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>215</v>
+        <v>199</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>215</v>
+        <v>199</v>
       </c>
       <c r="E6" s="1">
         <v>14</v>
@@ -3531,10 +3537,10 @@
         <v>2</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>215</v>
+        <v>199</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>215</v>
+        <v>199</v>
       </c>
       <c r="E7" s="1">
         <v>15</v>

</xml_diff>